<commit_message>
Refresh Excel reports from today's fully-passing GitHub Actions runs
All three suites are green on real CI infrastructure after the
backend-tests/DB-isolation/Selenium-warm-up changes:
- Backend Tests (Pytest) run 33905477547 — 8/8 passed
- Web E2E (Selenium) run 33905477597 — 17/17 passed (confirms the
  ChromeDriver warm-up fix; this run's "Landing page" spec, which used to
  intermittently time out, passed cleanly)
- Mobile E2E (Appium) run 33905481129 (rerun after an unrelated,
  self-resolving flake in the reactivecircus/android-emulator-runner
  action's own post-boot adb unlock step, before any of our test code
  ran) — 15/15 passed on a real Android emulator

Reports downloaded directly from these run artifacts, not regenerated
locally.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/appium-mobile/reports/appium-report.xlsx
+++ b/appium-mobile/reports/appium-report.xlsx
@@ -137,7 +137,7 @@
     <t>Run date</t>
   </si>
   <si>
-    <t>2026-09-04T07:31:20.300Z</t>
+    <t>2026-09-04T18:38:21.347Z</t>
   </si>
   <si>
     <t>By category</t>
@@ -586,7 +586,7 @@
         <v>8</v>
       </c>
       <c r="E2">
-        <v>6265</v>
+        <v>6068</v>
       </c>
       <c r="F2" t="s">
         <v>9</v>
@@ -606,7 +606,7 @@
         <v>8</v>
       </c>
       <c r="E3">
-        <v>3362</v>
+        <v>1387</v>
       </c>
       <c r="F3" t="s">
         <v>9</v>
@@ -626,7 +626,7 @@
         <v>8</v>
       </c>
       <c r="E4">
-        <v>51312</v>
+        <v>38683</v>
       </c>
       <c r="F4" t="s">
         <v>9</v>
@@ -646,7 +646,7 @@
         <v>8</v>
       </c>
       <c r="E5">
-        <v>21865</v>
+        <v>21551</v>
       </c>
       <c r="F5" t="s">
         <v>9</v>
@@ -666,7 +666,7 @@
         <v>8</v>
       </c>
       <c r="E6">
-        <v>1453</v>
+        <v>1681</v>
       </c>
       <c r="F6" t="s">
         <v>9</v>
@@ -686,7 +686,7 @@
         <v>8</v>
       </c>
       <c r="E7">
-        <v>1622</v>
+        <v>1369</v>
       </c>
       <c r="F7" t="s">
         <v>9</v>
@@ -706,7 +706,7 @@
         <v>8</v>
       </c>
       <c r="E8">
-        <v>1380</v>
+        <v>1422</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -726,7 +726,7 @@
         <v>8</v>
       </c>
       <c r="E9">
-        <v>1094</v>
+        <v>1127</v>
       </c>
       <c r="F9" t="s">
         <v>9</v>
@@ -746,7 +746,7 @@
         <v>8</v>
       </c>
       <c r="E10">
-        <v>23305</v>
+        <v>23734</v>
       </c>
       <c r="F10" t="s">
         <v>9</v>
@@ -766,7 +766,7 @@
         <v>8</v>
       </c>
       <c r="E11">
-        <v>35889</v>
+        <v>37563</v>
       </c>
       <c r="F11" t="s">
         <v>9</v>
@@ -786,7 +786,7 @@
         <v>8</v>
       </c>
       <c r="E12">
-        <v>29964</v>
+        <v>25391</v>
       </c>
       <c r="F12" t="s">
         <v>9</v>
@@ -806,7 +806,7 @@
         <v>8</v>
       </c>
       <c r="E13">
-        <v>2311</v>
+        <v>2360</v>
       </c>
       <c r="F13" t="s">
         <v>9</v>
@@ -826,7 +826,7 @@
         <v>8</v>
       </c>
       <c r="E14">
-        <v>2469</v>
+        <v>2838</v>
       </c>
       <c r="F14" t="s">
         <v>9</v>
@@ -846,7 +846,7 @@
         <v>8</v>
       </c>
       <c r="E15">
-        <v>1404</v>
+        <v>1517</v>
       </c>
       <c r="F15" t="s">
         <v>9</v>
@@ -866,7 +866,7 @@
         <v>8</v>
       </c>
       <c r="E16">
-        <v>19747</v>
+        <v>18972</v>
       </c>
       <c r="F16" t="s">
         <v>9</v>
@@ -932,7 +932,7 @@
         <v>39</v>
       </c>
       <c r="B6">
-        <v>203442</v>
+        <v>185663</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>